<commit_message>
Adding updates to gitignore
</commit_message>
<xml_diff>
--- a/app/static/datasets.xlsx
+++ b/app/static/datasets.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kokul/Projects/GOMAP-enrich/app/static/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65EA4E26-E229-5B4E-8E8B-97D8B60D5B4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C00836FC-4BE9-DA41-9AAA-6992EA83A8ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{E467A60D-F69A-4F4A-9E6E-FC569BD129C9}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="8">
   <si>
     <t>Species</t>
   </si>
@@ -50,10 +50,16 @@
     <t>B73_v4</t>
   </si>
   <si>
-    <t>maize.B73.AGPv4.aggregate.gaf</t>
-  </si>
-  <si>
     <t>Assembly</t>
+  </si>
+  <si>
+    <t>maize.B73.AGPv4.aggregate.gaf.gz</t>
+  </si>
+  <si>
+    <t>3.1_Zea_mays_B73.MaizeGDB.CLEANED.gaf.gz</t>
+  </si>
+  <si>
+    <t>B73_v5</t>
   </si>
 </sst>
 </file>
@@ -425,10 +431,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7DBB0A96-91CA-984C-B37F-8D25BAD45885}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="39.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
@@ -436,7 +442,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C1" t="s">
         <v>2</v>
@@ -450,7 +456,18 @@
         <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>4</v>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>